<commit_message>
Keep Finalized/PAID claims with empty Latest Date Worked at the top
An empty Latest Date Worked now takes precedence over the Finalized/PAID
rule, so those 16 claims sit in the top group in deadline order. Read Me
wording updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 01 January.xlsx
+++ b/SPC26S1 - 01 January.xlsx
@@ -1925,7 +1925,7 @@
     <t>50 claims with a date of service in 2026-01 January, split into one sheet per specialty: BH, DME, GAE, ORTHO, US.</t>
   </si>
   <si>
-    <t>Every specialty sheet is sorted in three groups: claims with an empty Latest Date Worked (column K) at the top, then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim goes to the bottom even when its Latest Date Worked is empty). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
+    <t>Every specialty sheet is sorted in three groups: claims with an empty Latest Date Worked (column K) at the top, then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim with an empty Latest Date Worked stays in the top group). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
   </si>
   <si>
     <t>Deadline order within each group, with the colour band each row gets, counted on 19 September 2026:</t>
@@ -6772,37 +6772,37 @@
     </row>
     <row r="2" spans="1:40" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="4">
         <v>46135</v>
       </c>
       <c r="D2" s="5">
-        <v>548883662</v>
+        <v>548880209</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="F2" s="7">
-        <v>46041</v>
+        <v>46034</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>187</v>
+        <v>43</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>44</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>187</v>
+        <v>43</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="5">
         <f ca="1">IF($O2="","",$O2-TODAY())</f>
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="M2" s="5">
         <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
@@ -6813,7 +6813,7 @@
         <v>-49</v>
       </c>
       <c r="O2" s="7">
-        <v>46406</v>
+        <v>46399</v>
       </c>
       <c r="P2" s="6" t="s">
         <v>46</v>
@@ -6834,10 +6834,10 @@
         <v>48</v>
       </c>
       <c r="V2" s="6" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="W2" s="6" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="X2" s="6" t="s">
         <v>174</v>
@@ -6861,26 +6861,24 @@
         <v>0.87</v>
       </c>
       <c r="AE2" s="5">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="AF2" s="6" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AG2" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="AH2" s="6" t="s">
-        <v>176</v>
-      </c>
+      <c r="AH2" s="6"/>
       <c r="AI2" s="6"/>
       <c r="AJ2" s="5">
-        <v>551561155</v>
+        <v>566386933</v>
       </c>
       <c r="AK2" s="6" t="s">
         <v>178</v>
       </c>
       <c r="AL2" s="6" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="AM2" s="7">
         <v>46062</v>
@@ -6891,48 +6889,48 @@
     </row>
     <row r="3" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4">
-        <v>46099</v>
+        <v>46147</v>
       </c>
       <c r="D3" s="5">
-        <v>552345092</v>
+        <v>548873847</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="F3" s="7">
-        <v>46048</v>
+        <v>46041</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>44</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="5">
         <f ca="1">IF($O3="","",$O3-TODAY())</f>
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="M3" s="5">
         <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="N3" s="5">
         <f ca="1">IF($C3="","",$C3+120-TODAY())</f>
-        <v>-85</v>
+        <v>-37</v>
       </c>
       <c r="O3" s="7">
-        <v>46413</v>
+        <v>46406</v>
       </c>
       <c r="P3" s="6" t="s">
         <v>46</v>
@@ -6952,31 +6950,29 @@
       <c r="U3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V3" s="6" t="s">
-        <v>199</v>
-      </c>
+      <c r="V3" s="6"/>
       <c r="W3" s="6"/>
       <c r="X3" s="6"/>
       <c r="Y3" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z3" s="9">
-        <v>52944.639999999999</v>
+        <v>49162.82</v>
       </c>
       <c r="AA3" s="9">
-        <v>3692.6</v>
+        <v>48759.59</v>
       </c>
       <c r="AB3" s="9">
-        <v>89.13</v>
+        <v>233.16</v>
       </c>
       <c r="AC3" s="7">
-        <v>46099</v>
+        <v>46147</v>
       </c>
       <c r="AD3" s="9">
-        <v>49162.91</v>
+        <v>170.07</v>
       </c>
       <c r="AE3" s="5">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="AF3" s="6" t="s">
         <v>184</v>
@@ -6987,11 +6983,9 @@
       <c r="AH3" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="AI3" s="6" t="s">
-        <v>200</v>
-      </c>
+      <c r="AI3" s="6"/>
       <c r="AJ3" s="5">
-        <v>551630154</v>
+        <v>565292656</v>
       </c>
       <c r="AK3" s="6" t="s">
         <v>178</v>
@@ -7000,100 +6994,104 @@
         <v>185</v>
       </c>
       <c r="AM3" s="7">
-        <v>46063</v>
+        <v>46062</v>
       </c>
       <c r="AN3" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:40" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
+    <row r="4" spans="1:40" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4">
-        <v>46121</v>
+        <v>46135</v>
       </c>
       <c r="D4" s="5">
-        <v>548877808</v>
+        <v>548883662</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="F4" s="7">
-        <v>46027</v>
+        <v>46041</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>202</v>
+        <v>44</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>76</v>
+        <v>187</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="5">
         <f ca="1">IF($O4="","",$O4-TODAY())</f>
-        <v>-187</v>
+        <v>102</v>
       </c>
       <c r="M4" s="5">
-        <f ca="1">IF($F4="","",$F4+90-TODAY())</f>
-        <v>-187</v>
+        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <v>196</v>
       </c>
       <c r="N4" s="5">
-        <f ca="1">IF($C4="","",$C4+540-TODAY())</f>
-        <v>357</v>
+        <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
+        <v>-49</v>
       </c>
       <c r="O4" s="7">
-        <v>46117</v>
+        <v>46406</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>204</v>
+        <v>47</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>303</v>
+        <v>49</v>
       </c>
       <c r="U4" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="W4" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="X4" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="X4" s="6"/>
       <c r="Y4" s="6" t="s">
         <v>175</v>
       </c>
       <c r="Z4" s="9">
-        <v>65892.820000000007</v>
+        <v>67599.91</v>
       </c>
       <c r="AA4" s="9">
-        <v>0</v>
+        <v>66731.289999999994</v>
       </c>
       <c r="AB4" s="9">
-        <v>0</v>
+        <v>867.75</v>
       </c>
       <c r="AC4" s="7">
-        <v>46121</v>
+        <v>46135</v>
       </c>
       <c r="AD4" s="9">
-        <v>65892.820000000007</v>
+        <v>0.87</v>
       </c>
       <c r="AE4" s="5">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="AF4" s="6" t="s">
         <v>184</v>
@@ -7105,7 +7103,9 @@
         <v>176</v>
       </c>
       <c r="AI4" s="6"/>
-      <c r="AJ4" s="5"/>
+      <c r="AJ4" s="5">
+        <v>551561155</v>
+      </c>
       <c r="AK4" s="6" t="s">
         <v>178</v>
       </c>
@@ -7119,94 +7119,98 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:40" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
+    <row r="5" spans="1:40" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4">
-        <v>46142</v>
+        <v>46120</v>
       </c>
       <c r="D5" s="5">
-        <v>554116779</v>
+        <v>548916508</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="F5" s="7">
-        <v>46027</v>
+        <v>46041</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>202</v>
+        <v>44</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>76</v>
+        <v>192</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="5">
         <f ca="1">IF($O5="","",$O5-TODAY())</f>
-        <v>-187</v>
+        <v>102</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($F5="","",$F5+90-TODAY())</f>
-        <v>-187</v>
+        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <v>181</v>
       </c>
       <c r="N5" s="5">
-        <f ca="1">IF($C5="","",$C5+540-TODAY())</f>
-        <v>378</v>
+        <f ca="1">IF($C5="","",$C5+120-TODAY())</f>
+        <v>-64</v>
       </c>
       <c r="O5" s="7">
-        <v>46117</v>
+        <v>46406</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>204</v>
+        <v>47</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>303</v>
+        <v>49</v>
       </c>
       <c r="U5" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="W5" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="X5" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="X5" s="6"/>
       <c r="Y5" s="6" t="s">
-        <v>115</v>
+        <v>175</v>
       </c>
       <c r="Z5" s="9">
-        <v>65085.23</v>
+        <v>67599.91</v>
       </c>
       <c r="AA5" s="9">
-        <v>0</v>
+        <v>66555.62</v>
       </c>
       <c r="AB5" s="9">
-        <v>0</v>
+        <v>867.75</v>
       </c>
       <c r="AC5" s="7">
-        <v>46142</v>
+        <v>46120</v>
       </c>
       <c r="AD5" s="9">
-        <v>65085.23</v>
+        <v>176.54</v>
       </c>
       <c r="AE5" s="5">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="AF5" s="6" t="s">
         <v>184</v>
@@ -7218,7 +7222,9 @@
         <v>176</v>
       </c>
       <c r="AI5" s="6"/>
-      <c r="AJ5" s="5"/>
+      <c r="AJ5" s="5">
+        <v>565292638</v>
+      </c>
       <c r="AK5" s="6" t="s">
         <v>178</v>
       </c>
@@ -7232,91 +7238,95 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:40" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
+    <row r="6" spans="1:40" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4">
-        <v>46111</v>
+        <v>46120</v>
       </c>
       <c r="D6" s="5">
-        <v>552170540</v>
+        <v>548917446</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="F6" s="7">
         <v>46048</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>202</v>
+        <v>149</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>202</v>
+        <v>44</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>76</v>
+        <v>149</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="5">
         <f ca="1">IF($O6="","",$O6-TODAY())</f>
-        <v>-166</v>
+        <v>109</v>
       </c>
       <c r="M6" s="5">
-        <f ca="1">IF($F6="","",$F6+90-TODAY())</f>
-        <v>-166</v>
+        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <v>181</v>
       </c>
       <c r="N6" s="5">
-        <f ca="1">IF($C6="","",$C6+540-TODAY())</f>
-        <v>347</v>
+        <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
+        <v>-64</v>
       </c>
       <c r="O6" s="7">
-        <v>46138</v>
+        <v>46413</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>204</v>
+        <v>47</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>303</v>
+        <v>49</v>
       </c>
       <c r="U6" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V6" s="6" t="s">
-        <v>205</v>
+        <v>172</v>
       </c>
       <c r="W6" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="X6" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="X6" s="6"/>
       <c r="Y6" s="6" t="s">
-        <v>59</v>
+        <v>196</v>
       </c>
       <c r="Z6" s="9">
-        <v>64277.64</v>
+        <v>21394.87</v>
       </c>
       <c r="AA6" s="9">
-        <v>0</v>
+        <v>20631.18</v>
       </c>
       <c r="AB6" s="9">
-        <v>0</v>
+        <v>506.12</v>
       </c>
       <c r="AC6" s="7">
-        <v>46111</v>
+        <v>46120</v>
       </c>
       <c r="AD6" s="9">
-        <v>64277.64</v>
+        <v>257.57</v>
       </c>
       <c r="AE6" s="5">
         <v>194</v>
@@ -7331,7 +7341,9 @@
         <v>176</v>
       </c>
       <c r="AI6" s="6"/>
-      <c r="AJ6" s="5"/>
+      <c r="AJ6" s="5">
+        <v>565292666</v>
+      </c>
       <c r="AK6" s="6" t="s">
         <v>178</v>
       </c>
@@ -7346,93 +7358,93 @@
       </c>
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4">
-        <v>46127</v>
+        <v>46099</v>
       </c>
       <c r="D7" s="5">
-        <v>555373347</v>
+        <v>552345092</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>210</v>
+        <v>197</v>
       </c>
       <c r="F7" s="7">
-        <v>46027</v>
+        <v>46048</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>211</v>
+        <v>145</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>211</v>
+        <v>44</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>76</v>
+        <v>145</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="5">
         <f ca="1">IF($O7="","",$O7-TODAY())</f>
-        <v>-157</v>
+        <v>109</v>
       </c>
       <c r="M7" s="5">
-        <f ca="1">IF($C7="","",$C7+180-TODAY())</f>
-        <v>3</v>
+        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <v>160</v>
       </c>
       <c r="N7" s="5">
-        <f ca="1">IF($C7="","",$C7+180-TODAY())</f>
-        <v>3</v>
+        <f ca="1">IF($C7="","",$C7+120-TODAY())</f>
+        <v>-85</v>
       </c>
       <c r="O7" s="7">
-        <v>46147</v>
+        <v>46413</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>213</v>
+        <v>47</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="S7" s="6" t="s">
         <v>48</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="U7" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="W7" s="6" t="s">
-        <v>174</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="W7" s="6"/>
       <c r="X7" s="6"/>
       <c r="Y7" s="6" t="s">
-        <v>214</v>
+        <v>59</v>
       </c>
       <c r="Z7" s="9">
-        <v>57326.78</v>
+        <v>52944.639999999999</v>
       </c>
       <c r="AA7" s="9">
-        <v>0</v>
+        <v>3692.6</v>
       </c>
       <c r="AB7" s="9">
-        <v>0</v>
+        <v>89.13</v>
       </c>
       <c r="AC7" s="7">
-        <v>46127</v>
+        <v>46099</v>
       </c>
       <c r="AD7" s="9">
-        <v>57326.78</v>
+        <v>49162.91</v>
       </c>
       <c r="AE7" s="5">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="AF7" s="6" t="s">
         <v>184</v>
@@ -7443,16 +7455,20 @@
       <c r="AH7" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="AI7" s="6"/>
-      <c r="AJ7" s="5"/>
+      <c r="AI7" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="AJ7" s="5">
+        <v>551630154</v>
+      </c>
       <c r="AK7" s="6" t="s">
         <v>178</v>
       </c>
       <c r="AL7" s="6" t="s">
-        <v>62</v>
+        <v>185</v>
       </c>
       <c r="AM7" s="7">
-        <v>46062</v>
+        <v>46063</v>
       </c>
       <c r="AN7" s="6" t="s">
         <v>180</v>
@@ -7462,64 +7478,75 @@
       <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="4">
-        <v>46141</v>
+        <v>46121</v>
       </c>
       <c r="D8" s="5">
-        <v>548926996</v>
+        <v>548877808</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="F8" s="7">
-        <v>46034</v>
+        <v>46027</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>217</v>
+        <v>76</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="K8" s="4"/>
-      <c r="L8" s="5" t="str">
+      <c r="L8" s="5">
         <f ca="1">IF($O8="","",$O8-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M8" s="5"/>
+        <v>-187</v>
+      </c>
+      <c r="M8" s="5">
+        <f ca="1">IF($F8="","",$F8+90-TODAY())</f>
+        <v>-187</v>
+      </c>
       <c r="N8" s="5">
-        <f ca="1">IF($C8="","",$C8+180-TODAY())</f>
-        <v>17</v>
-      </c>
-      <c r="O8" s="7"/>
-      <c r="P8" s="6"/>
+        <f ca="1">IF($C8="","",$C8+540-TODAY())</f>
+        <v>357</v>
+      </c>
+      <c r="O8" s="7">
+        <v>46117</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="Q8" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
+        <v>204</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>124</v>
+      </c>
       <c r="T8" s="6" t="s">
-        <v>80</v>
+        <v>303</v>
       </c>
       <c r="U8" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="W8" s="6" t="s">
         <v>174</v>
       </c>
       <c r="X8" s="6"/>
       <c r="Y8" s="6" t="s">
-        <v>221</v>
+        <v>175</v>
       </c>
       <c r="Z8" s="9">
-        <v>70557.69</v>
+        <v>65892.820000000007</v>
       </c>
       <c r="AA8" s="9">
         <v>0</v>
@@ -7528,13 +7555,13 @@
         <v>0</v>
       </c>
       <c r="AC8" s="7">
-        <v>46141</v>
+        <v>46121</v>
       </c>
       <c r="AD8" s="9">
-        <v>70557.69</v>
+        <v>65892.820000000007</v>
       </c>
       <c r="AE8" s="5">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="AF8" s="6" t="s">
         <v>184</v>
@@ -7551,7 +7578,7 @@
         <v>178</v>
       </c>
       <c r="AL8" s="6" t="s">
-        <v>90</v>
+        <v>185</v>
       </c>
       <c r="AM8" s="7">
         <v>46062</v>
@@ -7560,115 +7587,111 @@
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:40" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>94</v>
-      </c>
+    <row r="9" spans="1:40" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
       <c r="B9" s="3"/>
       <c r="C9" s="4">
-        <v>46135</v>
+        <v>46142</v>
       </c>
       <c r="D9" s="5">
-        <v>548880209</v>
+        <v>554116779</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>170</v>
+        <v>206</v>
       </c>
       <c r="F9" s="7">
-        <v>46034</v>
+        <v>46027</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>43</v>
+        <v>202</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>44</v>
+        <v>202</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="5">
         <f ca="1">IF($O9="","",$O9-TODAY())</f>
-        <v>95</v>
+        <v>-187</v>
       </c>
       <c r="M9" s="5">
-        <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
-        <v>196</v>
+        <f ca="1">IF($F9="","",$F9+90-TODAY())</f>
+        <v>-187</v>
       </c>
       <c r="N9" s="5">
-        <f ca="1">IF($C9="","",$C9+120-TODAY())</f>
-        <v>-49</v>
+        <f ca="1">IF($C9="","",$C9+540-TODAY())</f>
+        <v>378</v>
       </c>
       <c r="O9" s="7">
-        <v>46399</v>
+        <v>46117</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>47</v>
+        <v>204</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>49</v>
+        <v>303</v>
       </c>
       <c r="U9" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>172</v>
+        <v>205</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="X9" s="6" t="s">
         <v>174</v>
       </c>
+      <c r="X9" s="6"/>
       <c r="Y9" s="6" t="s">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="Z9" s="9">
-        <v>67599.91</v>
+        <v>65085.23</v>
       </c>
       <c r="AA9" s="9">
-        <v>66731.289999999994</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="9">
-        <v>867.75</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="7">
-        <v>46135</v>
+        <v>46142</v>
       </c>
       <c r="AD9" s="9">
-        <v>0.87</v>
+        <v>65085.23</v>
       </c>
       <c r="AE9" s="5">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="AF9" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="AG9" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="AH9" s="6"/>
+      <c r="AH9" s="6" t="s">
+        <v>176</v>
+      </c>
       <c r="AI9" s="6"/>
-      <c r="AJ9" s="5">
-        <v>566386933</v>
-      </c>
+      <c r="AJ9" s="5"/>
       <c r="AK9" s="6" t="s">
         <v>178</v>
       </c>
       <c r="AL9" s="6" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AM9" s="7">
         <v>46062</v>
@@ -7677,92 +7700,94 @@
         <v>180</v>
       </c>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>94</v>
-      </c>
+    <row r="10" spans="1:40" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
       <c r="B10" s="3"/>
       <c r="C10" s="4">
-        <v>46147</v>
+        <v>46111</v>
       </c>
       <c r="D10" s="5">
-        <v>548873847</v>
+        <v>552170540</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>181</v>
+        <v>208</v>
       </c>
       <c r="F10" s="7">
-        <v>46041</v>
+        <v>46048</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>44</v>
+        <v>202</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>182</v>
+        <v>76</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="5">
         <f ca="1">IF($O10="","",$O10-TODAY())</f>
-        <v>102</v>
+        <v>-166</v>
       </c>
       <c r="M10" s="5">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>208</v>
+        <f ca="1">IF($F10="","",$F10+90-TODAY())</f>
+        <v>-166</v>
       </c>
       <c r="N10" s="5">
-        <f ca="1">IF($C10="","",$C10+120-TODAY())</f>
-        <v>-37</v>
+        <f ca="1">IF($C10="","",$C10+540-TODAY())</f>
+        <v>347</v>
       </c>
       <c r="O10" s="7">
-        <v>46406</v>
+        <v>46138</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>47</v>
+        <v>204</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>49</v>
+        <v>303</v>
       </c>
       <c r="U10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6"/>
+      <c r="V10" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="W10" s="6" t="s">
+        <v>174</v>
+      </c>
       <c r="X10" s="6"/>
       <c r="Y10" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z10" s="9">
-        <v>49162.82</v>
+        <v>64277.64</v>
       </c>
       <c r="AA10" s="9">
-        <v>48759.59</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="9">
-        <v>233.16</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="7">
-        <v>46147</v>
+        <v>46111</v>
       </c>
       <c r="AD10" s="9">
-        <v>170.07</v>
+        <v>64277.64</v>
       </c>
       <c r="AE10" s="5">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="AF10" s="6" t="s">
         <v>184</v>
@@ -7774,9 +7799,7 @@
         <v>176</v>
       </c>
       <c r="AI10" s="6"/>
-      <c r="AJ10" s="5">
-        <v>565292656</v>
-      </c>
+      <c r="AJ10" s="5"/>
       <c r="AK10" s="6" t="s">
         <v>178</v>
       </c>
@@ -7790,98 +7813,94 @@
         <v>180</v>
       </c>
     </row>
-    <row r="11" spans="1:40" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>94</v>
-      </c>
+    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
       <c r="B11" s="3"/>
       <c r="C11" s="4">
-        <v>46120</v>
+        <v>46127</v>
       </c>
       <c r="D11" s="5">
-        <v>548916508</v>
+        <v>555373347</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="F11" s="7">
-        <v>46041</v>
+        <v>46027</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>44</v>
+        <v>211</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>192</v>
+        <v>76</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="5">
         <f ca="1">IF($O11="","",$O11-TODAY())</f>
-        <v>102</v>
+        <v>-157</v>
       </c>
       <c r="M11" s="5">
-        <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
-        <v>181</v>
+        <f ca="1">IF($C11="","",$C11+180-TODAY())</f>
+        <v>3</v>
       </c>
       <c r="N11" s="5">
-        <f ca="1">IF($C11="","",$C11+120-TODAY())</f>
-        <v>-64</v>
+        <f ca="1">IF($C11="","",$C11+180-TODAY())</f>
+        <v>3</v>
       </c>
       <c r="O11" s="7">
-        <v>46406</v>
+        <v>46147</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>47</v>
+        <v>213</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="S11" s="6" t="s">
         <v>48</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="U11" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="X11" s="6" t="s">
         <v>174</v>
       </c>
+      <c r="X11" s="6"/>
       <c r="Y11" s="6" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="Z11" s="9">
-        <v>67599.91</v>
+        <v>57326.78</v>
       </c>
       <c r="AA11" s="9">
-        <v>66555.62</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="9">
-        <v>867.75</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="7">
-        <v>46120</v>
+        <v>46127</v>
       </c>
       <c r="AD11" s="9">
-        <v>176.54</v>
+        <v>57326.78</v>
       </c>
       <c r="AE11" s="5">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="AF11" s="6" t="s">
         <v>184</v>
@@ -7893,14 +7912,12 @@
         <v>176</v>
       </c>
       <c r="AI11" s="6"/>
-      <c r="AJ11" s="5">
-        <v>565292638</v>
-      </c>
+      <c r="AJ11" s="5"/>
       <c r="AK11" s="6" t="s">
         <v>178</v>
       </c>
       <c r="AL11" s="6" t="s">
-        <v>185</v>
+        <v>62</v>
       </c>
       <c r="AM11" s="7">
         <v>46062</v>
@@ -7909,98 +7926,83 @@
         <v>180</v>
       </c>
     </row>
-    <row r="12" spans="1:40" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>94</v>
-      </c>
+    <row r="12" spans="1:40" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
       <c r="B12" s="3"/>
       <c r="C12" s="4">
-        <v>46120</v>
+        <v>46141</v>
       </c>
       <c r="D12" s="5">
-        <v>548917446</v>
+        <v>548926996</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="F12" s="7">
-        <v>46048</v>
+        <v>46034</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>44</v>
+        <v>216</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>149</v>
+        <v>217</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="K12" s="4"/>
-      <c r="L12" s="5">
+      <c r="L12" s="5" t="str">
         <f ca="1">IF($O12="","",$O12-TODAY())</f>
-        <v>109</v>
-      </c>
-      <c r="M12" s="5">
-        <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
-        <v>181</v>
-      </c>
+        <v/>
+      </c>
+      <c r="M12" s="5"/>
       <c r="N12" s="5">
-        <f ca="1">IF($C12="","",$C12+120-TODAY())</f>
-        <v>-64</v>
-      </c>
-      <c r="O12" s="7">
-        <v>46413</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>46</v>
-      </c>
+        <f ca="1">IF($C12="","",$C12+180-TODAY())</f>
+        <v>17</v>
+      </c>
+      <c r="O12" s="7"/>
+      <c r="P12" s="6"/>
       <c r="Q12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="R12" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="S12" s="6" t="s">
-        <v>48</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
       <c r="T12" s="6" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="U12" s="6" t="s">
         <v>48</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="X12" s="6" t="s">
         <v>174</v>
       </c>
+      <c r="X12" s="6"/>
       <c r="Y12" s="6" t="s">
-        <v>196</v>
+        <v>221</v>
       </c>
       <c r="Z12" s="9">
-        <v>21394.87</v>
+        <v>70557.69</v>
       </c>
       <c r="AA12" s="9">
-        <v>20631.18</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="9">
-        <v>506.12</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="7">
-        <v>46120</v>
+        <v>46141</v>
       </c>
       <c r="AD12" s="9">
-        <v>257.57</v>
+        <v>70557.69</v>
       </c>
       <c r="AE12" s="5">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="AF12" s="6" t="s">
         <v>184</v>
@@ -8012,14 +8014,12 @@
         <v>176</v>
       </c>
       <c r="AI12" s="6"/>
-      <c r="AJ12" s="5">
-        <v>565292666</v>
-      </c>
+      <c r="AJ12" s="5"/>
       <c r="AK12" s="6" t="s">
         <v>178</v>
       </c>
       <c r="AL12" s="6" t="s">
-        <v>185</v>
+        <v>90</v>
       </c>
       <c r="AM12" s="7">
         <v>46062</v>
@@ -8509,53 +8509,55 @@
       </c>
     </row>
     <row r="4" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
+      <c r="A4" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4">
-        <v>46045</v>
+        <v>46156</v>
       </c>
       <c r="D4" s="5">
-        <v>546049607</v>
+        <v>545934840</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F4" s="7">
-        <v>46035</v>
+        <v>46031</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>232</v>
       </c>
       <c r="H4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="J4" s="8" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="5">
         <f ca="1">IF($O4="","",$O4-TODAY())</f>
-        <v>-179</v>
+        <v>-183</v>
       </c>
       <c r="M4" s="5">
         <f ca="1">IF($C4="","",$C4+180-TODAY())</f>
-        <v>-79</v>
+        <v>32</v>
       </c>
       <c r="N4" s="5">
         <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
-        <v>106</v>
+        <v>217</v>
       </c>
       <c r="O4" s="7">
-        <v>46125</v>
+        <v>46121</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>236</v>
+        <v>79</v>
       </c>
       <c r="R4" s="6" t="s">
         <v>80</v>
@@ -8569,41 +8571,41 @@
       <c r="U4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V4" s="6" t="s">
-        <v>237</v>
-      </c>
+      <c r="V4" s="6"/>
       <c r="W4" s="6"/>
       <c r="X4" s="6"/>
       <c r="Y4" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z4" s="9">
-        <v>7623.07</v>
+        <v>2493.33</v>
       </c>
       <c r="AA4" s="9">
-        <v>0</v>
+        <v>2322.61</v>
       </c>
       <c r="AB4" s="9">
-        <v>0</v>
+        <v>18.5</v>
       </c>
       <c r="AC4" s="7">
-        <v>46045</v>
+        <v>46156</v>
       </c>
       <c r="AD4" s="9">
-        <v>7623.07</v>
+        <v>152.22</v>
       </c>
       <c r="AE4" s="5">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="AF4" s="6" t="s">
-        <v>141</v>
+        <v>233</v>
       </c>
       <c r="AG4" s="6"/>
       <c r="AH4" s="6"/>
       <c r="AI4" s="6"/>
-      <c r="AJ4" s="5"/>
+      <c r="AJ4" s="5">
+        <v>556916920</v>
+      </c>
       <c r="AK4" s="6" t="s">
-        <v>238</v>
+        <v>101</v>
       </c>
       <c r="AL4" s="6" t="s">
         <v>185</v>
@@ -8618,55 +8620,57 @@
     <row r="5" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
+      <c r="C5" s="4">
+        <v>46045</v>
+      </c>
       <c r="D5" s="5">
-        <v>548591390</v>
+        <v>546049607</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="F5" s="7">
-        <v>46036</v>
+        <v>46035</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>43</v>
+        <v>232</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>43</v>
+        <v>232</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="5">
         <f ca="1">IF($O5="","",$O5-TODAY())</f>
-        <v>-178</v>
+        <v>-179</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($F5="","",$F5+90-TODAY())</f>
-        <v>-178</v>
-      </c>
-      <c r="N5" s="5" t="str">
+        <f ca="1">IF($C5="","",$C5+180-TODAY())</f>
+        <v>-79</v>
+      </c>
+      <c r="N5" s="5">
         <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
-        <v/>
+        <v>106</v>
       </c>
       <c r="O5" s="7">
-        <v>46126</v>
+        <v>46125</v>
       </c>
       <c r="P5" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T5" s="6" t="s">
         <v>46</v>
@@ -8674,7 +8678,9 @@
       <c r="U5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V5" s="6"/>
+      <c r="V5" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="W5" s="6"/>
       <c r="X5" s="6"/>
       <c r="Y5" s="6" t="s">
@@ -8689,79 +8695,75 @@
       <c r="AB5" s="9">
         <v>0</v>
       </c>
-      <c r="AC5" s="7"/>
+      <c r="AC5" s="7">
+        <v>46045</v>
+      </c>
       <c r="AD5" s="9">
         <v>7623.07</v>
       </c>
       <c r="AE5" s="5">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AF5" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="AG5" s="6" t="s">
-        <v>133</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="AG5" s="6"/>
       <c r="AH5" s="6"/>
       <c r="AI5" s="6"/>
       <c r="AJ5" s="5"/>
       <c r="AK5" s="6" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="AL5" s="6" t="s">
         <v>185</v>
       </c>
       <c r="AM5" s="7">
-        <v>46042</v>
+        <v>46037</v>
       </c>
       <c r="AN5" s="6" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="A6" s="2"/>
       <c r="B6" s="3"/>
-      <c r="C6" s="4">
-        <v>46163</v>
-      </c>
+      <c r="C6" s="4"/>
       <c r="D6" s="5">
-        <v>547275123</v>
+        <v>548591390</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F6" s="7">
-        <v>46045</v>
+        <v>46036</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>43</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="5">
         <f ca="1">IF($O6="","",$O6-TODAY())</f>
-        <v>-169</v>
+        <v>-178</v>
       </c>
       <c r="M6" s="5">
         <f ca="1">IF($F6="","",$F6+90-TODAY())</f>
-        <v>-169</v>
-      </c>
-      <c r="N6" s="5">
+        <v>-178</v>
+      </c>
+      <c r="N6" s="5" t="str">
         <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>224</v>
+        <v/>
       </c>
       <c r="O6" s="7">
-        <v>46135</v>
+        <v>46126</v>
       </c>
       <c r="P6" s="6" t="s">
         <v>78</v>
@@ -8781,49 +8783,45 @@
       <c r="U6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V6" s="6" t="s">
-        <v>237</v>
-      </c>
+      <c r="V6" s="6"/>
       <c r="W6" s="6"/>
       <c r="X6" s="6"/>
       <c r="Y6" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z6" s="9">
-        <v>5614.63</v>
+        <v>7623.07</v>
       </c>
       <c r="AA6" s="9">
-        <v>-186.91</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <v>0</v>
       </c>
-      <c r="AC6" s="7">
-        <v>46163</v>
-      </c>
+      <c r="AC6" s="7"/>
       <c r="AD6" s="9">
-        <v>5614.63</v>
+        <v>7623.07</v>
       </c>
       <c r="AE6" s="5">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="AF6" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="AG6" s="6"/>
+        <v>240</v>
+      </c>
+      <c r="AG6" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="AH6" s="6"/>
       <c r="AI6" s="6"/>
-      <c r="AJ6" s="5">
-        <v>549237390</v>
-      </c>
+      <c r="AJ6" s="5"/>
       <c r="AK6" s="6" t="s">
-        <v>52</v>
+        <v>241</v>
       </c>
       <c r="AL6" s="6" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AM6" s="7">
-        <v>46049</v>
+        <v>46042</v>
       </c>
       <c r="AN6" s="6" t="s">
         <v>226</v>
@@ -8833,32 +8831,30 @@
       <c r="A7" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>245</v>
-      </c>
+      <c r="B7" s="3"/>
       <c r="C7" s="4">
-        <v>46052</v>
+        <v>46163</v>
       </c>
       <c r="D7" s="5">
-        <v>547576017</v>
+        <v>547275123</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="F7" s="7">
         <v>46045</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>43</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="5">
@@ -8871,7 +8867,7 @@
       </c>
       <c r="N7" s="5">
         <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
-        <v>113</v>
+        <v>224</v>
       </c>
       <c r="O7" s="7">
         <v>46135</v>
@@ -8894,42 +8890,46 @@
       <c r="U7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="V7" s="6"/>
+      <c r="V7" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="W7" s="6"/>
       <c r="X7" s="6"/>
       <c r="Y7" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z7" s="9">
-        <v>7623.07</v>
+        <v>5614.63</v>
       </c>
       <c r="AA7" s="9">
-        <v>0</v>
+        <v>-186.91</v>
       </c>
       <c r="AB7" s="9">
         <v>0</v>
       </c>
       <c r="AC7" s="7">
-        <v>46052</v>
+        <v>46163</v>
       </c>
       <c r="AD7" s="9">
-        <v>7623.07</v>
+        <v>5614.63</v>
       </c>
       <c r="AE7" s="5">
         <v>197</v>
       </c>
       <c r="AF7" s="6" t="s">
-        <v>141</v>
+        <v>244</v>
       </c>
       <c r="AG7" s="6"/>
       <c r="AH7" s="6"/>
       <c r="AI7" s="6"/>
-      <c r="AJ7" s="5"/>
+      <c r="AJ7" s="5">
+        <v>549237390</v>
+      </c>
       <c r="AK7" s="6" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="AL7" s="6" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="AM7" s="7">
         <v>46049</v>
@@ -8939,60 +8939,78 @@
       </c>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
+      <c r="A8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C8" s="4">
-        <v>46111</v>
+        <v>46052</v>
       </c>
       <c r="D8" s="5">
-        <v>549178846</v>
+        <v>547576017</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F8" s="7">
         <v>46045</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>248</v>
+        <v>43</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>248</v>
+        <v>43</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="K8" s="4"/>
-      <c r="L8" s="5" t="str">
+      <c r="L8" s="5">
         <f ca="1">IF($O8="","",$O8-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="6"/>
+        <v>-169</v>
+      </c>
+      <c r="M8" s="5">
+        <f ca="1">IF($F8="","",$F8+90-TODAY())</f>
+        <v>-169</v>
+      </c>
+      <c r="N8" s="5">
+        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
+        <v>113</v>
+      </c>
+      <c r="O8" s="7">
+        <v>46135</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="Q8" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="W8" s="6" t="s">
-        <v>205</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
       <c r="X8" s="6"/>
       <c r="Y8" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z8" s="9">
-        <v>3516.24</v>
+        <v>7623.07</v>
       </c>
       <c r="AA8" s="9">
         <v>0</v>
@@ -9001,31 +9019,29 @@
         <v>0</v>
       </c>
       <c r="AC8" s="7">
-        <v>46111</v>
+        <v>46052</v>
       </c>
       <c r="AD8" s="9">
-        <v>3516.24</v>
+        <v>7623.07</v>
       </c>
       <c r="AE8" s="5">
         <v>197</v>
       </c>
       <c r="AF8" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="AG8" s="6" t="s">
-        <v>133</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="AG8" s="6"/>
       <c r="AH8" s="6"/>
       <c r="AI8" s="6"/>
       <c r="AJ8" s="5"/>
       <c r="AK8" s="6" t="s">
-        <v>241</v>
+        <v>101</v>
       </c>
       <c r="AL8" s="6" t="s">
-        <v>253</v>
+        <v>185</v>
       </c>
       <c r="AM8" s="7">
-        <v>46058</v>
+        <v>46049</v>
       </c>
       <c r="AN8" s="6" t="s">
         <v>226</v>
@@ -9035,28 +9051,28 @@
       <c r="A9" s="2"/>
       <c r="B9" s="3"/>
       <c r="C9" s="4">
-        <v>46177</v>
+        <v>46111</v>
       </c>
       <c r="D9" s="5">
-        <v>557657640</v>
+        <v>549178846</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="F9" s="7">
-        <v>46048</v>
+        <v>46045</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="5" t="str">
@@ -9075,15 +9091,17 @@
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="W9" s="6"/>
+        <v>251</v>
+      </c>
+      <c r="W9" s="6" t="s">
+        <v>205</v>
+      </c>
       <c r="X9" s="6"/>
       <c r="Y9" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z9" s="9">
-        <v>5784.24</v>
+        <v>3516.24</v>
       </c>
       <c r="AA9" s="9">
         <v>0</v>
@@ -9092,120 +9110,104 @@
         <v>0</v>
       </c>
       <c r="AC9" s="7">
-        <v>46177</v>
+        <v>46111</v>
       </c>
       <c r="AD9" s="9">
-        <v>5784.24</v>
+        <v>3516.24</v>
       </c>
       <c r="AE9" s="5">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AF9" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="AG9" s="6"/>
+        <v>252</v>
+      </c>
+      <c r="AG9" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="AH9" s="6"/>
       <c r="AI9" s="6"/>
       <c r="AJ9" s="5"/>
       <c r="AK9" s="6" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="AL9" s="6" t="s">
-        <v>185</v>
+        <v>253</v>
       </c>
       <c r="AM9" s="7">
-        <v>46079</v>
+        <v>46058</v>
       </c>
       <c r="AN9" s="6" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>94</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" s="3"/>
       <c r="C10" s="4">
-        <v>46156</v>
+        <v>46177</v>
       </c>
       <c r="D10" s="5">
-        <v>545934840</v>
+        <v>557657640</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>231</v>
+        <v>254</v>
       </c>
       <c r="F10" s="7">
-        <v>46031</v>
+        <v>46048</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>232</v>
+        <v>255</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>75</v>
+        <v>255</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>232</v>
+        <v>76</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>224</v>
+        <v>256</v>
       </c>
       <c r="K10" s="4"/>
-      <c r="L10" s="5">
+      <c r="L10" s="5" t="str">
         <f ca="1">IF($O10="","",$O10-TODAY())</f>
-        <v>-183</v>
-      </c>
-      <c r="M10" s="5">
-        <f ca="1">IF($C10="","",$C10+180-TODAY())</f>
-        <v>32</v>
-      </c>
-      <c r="N10" s="5">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>217</v>
-      </c>
-      <c r="O10" s="7">
-        <v>46121</v>
-      </c>
-      <c r="P10" s="6" t="s">
-        <v>78</v>
-      </c>
+        <v/>
+      </c>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="6"/>
       <c r="Q10" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="R10" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="S10" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="T10" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="U10" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="V10" s="6"/>
+        <v>250</v>
+      </c>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6" t="s">
+        <v>257</v>
+      </c>
       <c r="W10" s="6"/>
       <c r="X10" s="6"/>
       <c r="Y10" s="6" t="s">
         <v>59</v>
       </c>
       <c r="Z10" s="9">
-        <v>2493.33</v>
+        <v>5784.24</v>
       </c>
       <c r="AA10" s="9">
-        <v>2322.61</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="9">
-        <v>18.5</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="7">
-        <v>46156</v>
+        <v>46177</v>
       </c>
       <c r="AD10" s="9">
-        <v>152.22</v>
+        <v>5784.24</v>
       </c>
       <c r="AE10" s="5">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="AF10" s="6" t="s">
         <v>233</v>
@@ -9213,17 +9215,15 @@
       <c r="AG10" s="6"/>
       <c r="AH10" s="6"/>
       <c r="AI10" s="6"/>
-      <c r="AJ10" s="5">
-        <v>556916920</v>
-      </c>
+      <c r="AJ10" s="5"/>
       <c r="AK10" s="6" t="s">
-        <v>101</v>
+        <v>258</v>
       </c>
       <c r="AL10" s="6" t="s">
         <v>185</v>
       </c>
       <c r="AM10" s="7">
-        <v>46037</v>
+        <v>46079</v>
       </c>
       <c r="AN10" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Move Rejected claims to the top of each monthly claim sheet
Order is now: Rejected, then empty Latest Date Worked, then other open
claims, then Finalized/PAID. Deadline order is kept within each group.
Read Me wording updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 01 January.xlsx
+++ b/SPC26S1 - 01 January.xlsx
@@ -1868,7 +1868,7 @@
     <t>Past due rows sit below the claims that can still be filed on time rather than at the very top, so the actionable work stays first. That is why the numbers run up to the longest window and then restart at the negatives.</t>
   </si>
   <si>
-    <t>Filing Deadline is the date of service plus the primary payer's limit, taken from 'Carrier_Timely_Filing_Reference.xlsx'. Days Until Deadline is a live formula, so the count stays true as time passes - but the row order is a snapshot taken on 12 August 2026. Sorting on Days Until Deadline alone would mix the three groups above back together, so when you re-sort keep the empty Latest Date Worked rows first and the Finalized and PAID rows last.</t>
+    <t>Filing Deadline is the date of service plus the primary payer's limit, taken from 'Carrier_Timely_Filing_Reference.xlsx'. Days Until Deadline is a live formula, so the count stays true as time passes - but the row order is a snapshot taken on 12 August 2026. Sorting on Days Until Deadline alone would mix the four groups above back together, so when you re-sort keep the Rejected rows first, then the empty Latest Date Worked rows, and the Finalized and PAID rows last.</t>
   </si>
   <si>
     <t>Where a payer had two possible limits the shorter one was used, so the real deadline can only be later, never earlier. Filing Limit and Limit Carrier name the figure applied and the carrier row it came from.</t>
@@ -1925,7 +1925,7 @@
     <t>50 claims with a date of service in 2026-01 January, split into one sheet per specialty: BH, DME, GAE, ORTHO, US.</t>
   </si>
   <si>
-    <t>Every specialty sheet is sorted in three groups: claims with an empty Latest Date Worked (column K) at the top, then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim with an empty Latest Date Worked stays in the top group). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
+    <t>Every specialty sheet is sorted in four groups: Rejected claims at the very top, then claims with an empty Latest Date Worked (column K), then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim with an empty Latest Date Worked stays in the empty Latest Date Worked group). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
   </si>
   <si>
     <t>Deadline order within each group, with the colour band each row gets, counted on 19 September 2026:</t>
@@ -3646,56 +3646,58 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>110</v>
       </c>
       <c r="C2" s="4">
-        <v>46071</v>
+        <v>46098</v>
       </c>
       <c r="D2" s="5">
-        <v>547309790</v>
+        <v>557090486</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="F2" s="7">
-        <v>46043</v>
+        <v>46036</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="K2" s="4"/>
+        <v>113</v>
+      </c>
+      <c r="K2" s="4">
+        <v>46135</v>
+      </c>
       <c r="L2" s="14">
         <f ca="1">IF($O2="","",$O2-TODAY())</f>
-        <v>104</v>
+        <v>-148</v>
       </c>
       <c r="M2" s="14">
         <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="N2" s="14">
-        <f ca="1">IF($C2="","",$C2+120-TODAY())</f>
-        <v>-113</v>
+        <f ca="1">IF($C2="","",$C2+90-TODAY())</f>
+        <v>-116</v>
       </c>
       <c r="O2" s="7">
-        <v>46408</v>
+        <v>46156</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>47</v>
+        <v>114</v>
       </c>
       <c r="R2" s="6" t="s">
         <v>46</v>
@@ -3704,7 +3706,7 @@
         <v>48</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="U2" s="6" t="s">
         <v>48</v>
@@ -3713,35 +3715,33 @@
       <c r="W2" s="6"/>
       <c r="X2" s="6"/>
       <c r="Y2" s="6" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="Z2" s="9">
-        <v>976.64</v>
+        <v>1769.18</v>
       </c>
       <c r="AA2" s="9">
-        <v>846.88</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="9">
-        <v>101.35</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="7">
-        <v>46071</v>
+        <v>46098</v>
       </c>
       <c r="AD2" s="9">
-        <v>28.41</v>
+        <v>1769.18</v>
       </c>
       <c r="AE2" s="5">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="AF2" s="6" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="AG2" s="6"/>
       <c r="AH2" s="6"/>
       <c r="AI2" s="6"/>
-      <c r="AJ2" s="5">
-        <v>550866344</v>
-      </c>
+      <c r="AJ2" s="5"/>
       <c r="AK2" s="6" t="s">
         <v>61</v>
       </c>
@@ -3757,54 +3757,58 @@
     </row>
     <row r="3" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="2"/>
+        <v>109</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>315</v>
+      </c>
       <c r="C3" s="4">
-        <v>46129</v>
+        <v>46070</v>
       </c>
       <c r="D3" s="5">
-        <v>555619522</v>
+        <v>565238310</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F3" s="7">
-        <v>46044</v>
+        <v>46045</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>44</v>
+        <v>118</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>44</v>
+        <v>118</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="K3" s="4"/>
+        <v>100</v>
+      </c>
+      <c r="K3" s="4">
+        <v>46289</v>
+      </c>
       <c r="L3" s="14">
         <f ca="1">IF($O3="","",$O3-TODAY())</f>
-        <v>105</v>
+        <v>-79</v>
       </c>
       <c r="M3" s="14">
         <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
-        <v>190</v>
+        <v>131</v>
       </c>
       <c r="N3" s="14">
-        <f ca="1">IF($C3="","",$C3+120-TODAY())</f>
-        <v>-55</v>
+        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <v>131</v>
       </c>
       <c r="O3" s="7">
-        <v>46409</v>
+        <v>46225</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>47</v>
+        <v>119</v>
       </c>
       <c r="R3" s="6" t="s">
         <v>46</v>
@@ -3813,7 +3817,7 @@
         <v>48</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="U3" s="6" t="s">
         <v>48</v>
@@ -3834,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="AC3" s="7">
-        <v>46129</v>
+        <v>46070</v>
       </c>
       <c r="AD3" s="9">
         <v>1426.25</v>
       </c>
       <c r="AE3" s="5">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AF3" s="6" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -3853,10 +3857,10 @@
         <v>67</v>
       </c>
       <c r="AL3" s="6" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="AM3" s="7">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="AN3" s="6" t="s">
         <v>54</v>
@@ -3867,28 +3871,28 @@
         <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="C4" s="4">
-        <v>46072</v>
+        <v>46071</v>
       </c>
       <c r="D4" s="5">
-        <v>547756234</v>
+        <v>547309790</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="F4" s="7">
-        <v>46050</v>
+        <v>46043</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>44</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>58</v>
@@ -3896,18 +3900,18 @@
       <c r="K4" s="4"/>
       <c r="L4" s="14">
         <f ca="1">IF($O4="","",$O4-TODAY())</f>
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="M4" s="14">
         <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N4" s="14">
         <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
-        <v>-112</v>
+        <v>-113</v>
       </c>
       <c r="O4" s="7">
-        <v>46415</v>
+        <v>46408</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>46</v>
@@ -3937,37 +3941,37 @@
         <v>976.64</v>
       </c>
       <c r="AA4" s="9">
-        <v>844.25</v>
+        <v>846.88</v>
       </c>
       <c r="AB4" s="9">
-        <v>103.98</v>
+        <v>101.35</v>
       </c>
       <c r="AC4" s="7">
-        <v>46072</v>
+        <v>46071</v>
       </c>
       <c r="AD4" s="9">
         <v>28.41</v>
       </c>
       <c r="AE4" s="5">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="AF4" s="6" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="AG4" s="6"/>
       <c r="AH4" s="6"/>
       <c r="AI4" s="6"/>
       <c r="AJ4" s="5">
-        <v>550865889</v>
+        <v>550866344</v>
       </c>
       <c r="AK4" s="6" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="AL4" s="6" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="AM4" s="7">
-        <v>46057</v>
+        <v>46056</v>
       </c>
       <c r="AN4" s="6" t="s">
         <v>54</v>
@@ -3977,29 +3981,27 @@
       <c r="A5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>317</v>
-      </c>
+      <c r="B5" s="2"/>
       <c r="C5" s="4">
-        <v>46063</v>
+        <v>46129</v>
       </c>
       <c r="D5" s="5">
-        <v>545484752</v>
+        <v>555619522</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="F5" s="7">
-        <v>46029</v>
+        <v>46044</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>66</v>
@@ -4007,33 +4009,33 @@
       <c r="K5" s="4"/>
       <c r="L5" s="14">
         <f ca="1">IF($O5="","",$O5-TODAY())</f>
-        <v>-185</v>
+        <v>105</v>
       </c>
       <c r="M5" s="14">
-        <f ca="1">IF($F5="","",$F5+90-TODAY())</f>
-        <v>-185</v>
+        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <v>190</v>
       </c>
       <c r="N5" s="14">
-        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
-        <v>124</v>
+        <f ca="1">IF($C5="","",$C5+120-TODAY())</f>
+        <v>-55</v>
       </c>
       <c r="O5" s="7">
-        <v>46119</v>
+        <v>46409</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="U5" s="6" t="s">
         <v>48</v>
@@ -4054,13 +4056,13 @@
         <v>0</v>
       </c>
       <c r="AC5" s="7">
-        <v>46063</v>
+        <v>46129</v>
       </c>
       <c r="AD5" s="9">
         <v>1426.25</v>
       </c>
       <c r="AE5" s="5">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="AF5" s="6" t="s">
         <v>51</v>
@@ -4070,13 +4072,13 @@
       <c r="AI5" s="6"/>
       <c r="AJ5" s="5"/>
       <c r="AK5" s="6" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="AL5" s="6" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="AM5" s="7">
-        <v>46057</v>
+        <v>46056</v>
       </c>
       <c r="AN5" s="6" t="s">
         <v>54</v>
@@ -4084,65 +4086,65 @@
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>317</v>
+        <v>68</v>
       </c>
       <c r="C6" s="4">
-        <v>46141</v>
+        <v>46072</v>
       </c>
       <c r="D6" s="5">
-        <v>545748574</v>
+        <v>547756234</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="F6" s="7">
-        <v>46031</v>
+        <v>46050</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="14">
         <f ca="1">IF($O6="","",$O6-TODAY())</f>
-        <v>-183</v>
+        <v>111</v>
       </c>
       <c r="M6" s="14">
-        <f ca="1">IF($C6="","",$C6+180-TODAY())</f>
-        <v>17</v>
+        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <v>133</v>
       </c>
       <c r="N6" s="14">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>202</v>
+        <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
+        <v>-112</v>
       </c>
       <c r="O6" s="7">
-        <v>46121</v>
+        <v>46415</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="S6" s="6" t="s">
         <v>48</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="U6" s="6" t="s">
         <v>48</v>
@@ -4154,32 +4156,34 @@
         <v>59</v>
       </c>
       <c r="Z6" s="9">
-        <v>1426.25</v>
+        <v>976.64</v>
       </c>
       <c r="AA6" s="9">
-        <v>0</v>
+        <v>844.25</v>
       </c>
       <c r="AB6" s="9">
-        <v>0</v>
+        <v>103.98</v>
       </c>
       <c r="AC6" s="7">
-        <v>46141</v>
+        <v>46072</v>
       </c>
       <c r="AD6" s="9">
-        <v>1426.25</v>
+        <v>28.41</v>
       </c>
       <c r="AE6" s="5">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="AF6" s="6" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
       <c r="AI6" s="6"/>
-      <c r="AJ6" s="5"/>
+      <c r="AJ6" s="5">
+        <v>550865889</v>
+      </c>
       <c r="AK6" s="6" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="AL6" s="6" t="s">
         <v>53</v>
@@ -4196,61 +4200,59 @@
         <v>63</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>73</v>
+        <v>317</v>
       </c>
       <c r="C7" s="4">
-        <v>46142</v>
+        <v>46063</v>
       </c>
       <c r="D7" s="5">
-        <v>545332485</v>
+        <v>545484752</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F7" s="7">
-        <v>46028</v>
+        <v>46029</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="K7" s="4">
-        <v>46122</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="K7" s="4"/>
       <c r="L7" s="14">
         <f ca="1">IF($O7="","",$O7-TODAY())</f>
-        <v>-186</v>
+        <v>-185</v>
       </c>
       <c r="M7" s="14">
-        <f ca="1">IF($C7="","",$C7+180-TODAY())</f>
-        <v>18</v>
+        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
+        <v>-185</v>
       </c>
       <c r="N7" s="14">
         <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
-        <v>203</v>
+        <v>124</v>
       </c>
       <c r="O7" s="7">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="P7" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="T7" s="6" t="s">
         <v>46</v>
@@ -4265,7 +4267,7 @@
         <v>59</v>
       </c>
       <c r="Z7" s="9">
-        <v>396.27</v>
+        <v>1426.25</v>
       </c>
       <c r="AA7" s="9">
         <v>0</v>
@@ -4274,13 +4276,13 @@
         <v>0</v>
       </c>
       <c r="AC7" s="7">
-        <v>46142</v>
+        <v>46063</v>
       </c>
       <c r="AD7" s="9">
-        <v>396.27</v>
+        <v>1426.25</v>
       </c>
       <c r="AE7" s="5">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AF7" s="6" t="s">
         <v>51</v>
@@ -4290,7 +4292,7 @@
       <c r="AI7" s="6"/>
       <c r="AJ7" s="5"/>
       <c r="AK7" s="6" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="AL7" s="6" t="s">
         <v>53</v>
@@ -4307,58 +4309,56 @@
         <v>63</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>85</v>
+        <v>317</v>
       </c>
       <c r="C8" s="4">
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="D8" s="5">
-        <v>556348109</v>
+        <v>545748574</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F8" s="7">
-        <v>46036</v>
+        <v>46031</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="K8" s="4">
-        <v>46129</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="K8" s="4"/>
       <c r="L8" s="14">
         <f ca="1">IF($O8="","",$O8-TODAY())</f>
-        <v>-178</v>
+        <v>-183</v>
       </c>
       <c r="M8" s="14">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
-        <v>194</v>
+        <f ca="1">IF($C8="","",$C8+180-TODAY())</f>
+        <v>17</v>
       </c>
       <c r="N8" s="14">
         <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="O8" s="7">
-        <v>46126</v>
+        <v>46121</v>
       </c>
       <c r="P8" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="S8" s="6" t="s">
         <v>48</v>
@@ -4376,7 +4376,7 @@
         <v>59</v>
       </c>
       <c r="Z8" s="9">
-        <v>976.64</v>
+        <v>1426.25</v>
       </c>
       <c r="AA8" s="9">
         <v>0</v>
@@ -4385,26 +4385,26 @@
         <v>0</v>
       </c>
       <c r="AC8" s="7">
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="AD8" s="9">
-        <v>976.64</v>
+        <v>1426.25</v>
       </c>
       <c r="AE8" s="5">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="AF8" s="6" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="AG8" s="6"/>
       <c r="AH8" s="6"/>
       <c r="AI8" s="6"/>
       <c r="AJ8" s="5"/>
       <c r="AK8" s="6" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="AL8" s="6" t="s">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="AM8" s="7">
         <v>46057</v>
@@ -4418,61 +4418,61 @@
         <v>63</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C9" s="4">
-        <v>46064</v>
+        <v>46142</v>
       </c>
       <c r="D9" s="5">
-        <v>548015539</v>
+        <v>545332485</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="F9" s="7">
-        <v>46043</v>
+        <v>46028</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="K9" s="4">
-        <v>46134</v>
+        <v>46122</v>
       </c>
       <c r="L9" s="14">
         <f ca="1">IF($O9="","",$O9-TODAY())</f>
-        <v>-171</v>
+        <v>-186</v>
       </c>
       <c r="M9" s="14">
-        <f ca="1">IF($F9="","",$F9+90-TODAY())</f>
-        <v>-171</v>
+        <f ca="1">IF($C9="","",$C9+180-TODAY())</f>
+        <v>18</v>
       </c>
       <c r="N9" s="14">
         <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
-        <v>125</v>
+        <v>203</v>
       </c>
       <c r="O9" s="7">
-        <v>46133</v>
+        <v>46118</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T9" s="6" t="s">
         <v>46</v>
@@ -4487,7 +4487,7 @@
         <v>59</v>
       </c>
       <c r="Z9" s="9">
-        <v>1426.25</v>
+        <v>396.27</v>
       </c>
       <c r="AA9" s="9">
         <v>0</v>
@@ -4496,26 +4496,26 @@
         <v>0</v>
       </c>
       <c r="AC9" s="7">
-        <v>46064</v>
+        <v>46142</v>
       </c>
       <c r="AD9" s="9">
-        <v>1426.25</v>
+        <v>396.27</v>
       </c>
       <c r="AE9" s="5">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="AF9" s="6" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="AG9" s="6"/>
       <c r="AH9" s="6"/>
       <c r="AI9" s="6"/>
       <c r="AJ9" s="5"/>
       <c r="AK9" s="6" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="AL9" s="6" t="s">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="AM9" s="7">
         <v>46057</v>
@@ -4526,64 +4526,64 @@
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>316</v>
+        <v>85</v>
       </c>
       <c r="C10" s="4">
-        <v>46094</v>
+        <v>46133</v>
       </c>
       <c r="D10" s="5">
-        <v>547442681</v>
+        <v>556348109</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F10" s="7">
-        <v>46044</v>
+        <v>46036</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>58</v>
       </c>
       <c r="K10" s="4">
-        <v>46304</v>
+        <v>46129</v>
       </c>
       <c r="L10" s="14">
         <f ca="1">IF($O10="","",$O10-TODAY())</f>
-        <v>-170</v>
+        <v>-178</v>
       </c>
       <c r="M10" s="14">
-        <f ca="1">IF($F10="","",$F10+90-TODAY())</f>
-        <v>-170</v>
+        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
+        <v>194</v>
       </c>
       <c r="N10" s="14">
         <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="O10" s="7">
-        <v>46134</v>
+        <v>46126</v>
       </c>
       <c r="P10" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="T10" s="6" t="s">
         <v>46</v>
@@ -4601,37 +4601,35 @@
         <v>976.64</v>
       </c>
       <c r="AA10" s="9">
-        <v>840.66</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="9">
         <v>0</v>
       </c>
       <c r="AC10" s="7">
-        <v>46094</v>
+        <v>46133</v>
       </c>
       <c r="AD10" s="9">
-        <v>135.97999999999999</v>
+        <v>976.64</v>
       </c>
       <c r="AE10" s="5">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="AF10" s="6" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="AG10" s="6"/>
       <c r="AH10" s="6"/>
       <c r="AI10" s="6"/>
-      <c r="AJ10" s="5">
-        <v>556556161</v>
-      </c>
+      <c r="AJ10" s="5"/>
       <c r="AK10" s="6" t="s">
         <v>52</v>
       </c>
       <c r="AL10" s="6" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="AM10" s="7">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="AN10" s="6" t="s">
         <v>54</v>
@@ -4639,22 +4637,22 @@
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C11" s="4">
-        <v>46128</v>
+        <v>46064</v>
       </c>
       <c r="D11" s="5">
-        <v>555599776</v>
+        <v>548015539</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="F11" s="7">
-        <v>46049</v>
+        <v>46043</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>43</v>
@@ -4663,28 +4661,28 @@
         <v>43</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="K11" s="4">
-        <v>46122</v>
+        <v>46134</v>
       </c>
       <c r="L11" s="14">
         <f ca="1">IF($O11="","",$O11-TODAY())</f>
-        <v>-165</v>
+        <v>-171</v>
       </c>
       <c r="M11" s="14">
         <f ca="1">IF($F11="","",$F11+90-TODAY())</f>
-        <v>-165</v>
+        <v>-171</v>
       </c>
       <c r="N11" s="14">
         <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
-        <v>189</v>
+        <v>125</v>
       </c>
       <c r="O11" s="7">
-        <v>46139</v>
+        <v>46133</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>78</v>
@@ -4720,26 +4718,26 @@
         <v>0</v>
       </c>
       <c r="AC11" s="7">
-        <v>46128</v>
+        <v>46064</v>
       </c>
       <c r="AD11" s="9">
         <v>1426.25</v>
       </c>
       <c r="AE11" s="5">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="AF11" s="6" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="AG11" s="6"/>
       <c r="AH11" s="6"/>
       <c r="AI11" s="6"/>
       <c r="AJ11" s="5"/>
       <c r="AK11" s="6" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="AL11" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="AM11" s="7">
         <v>46057</v>
@@ -4750,64 +4748,64 @@
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C12" s="4">
-        <v>46287</v>
+        <v>46094</v>
       </c>
       <c r="D12" s="5">
-        <v>556349314</v>
+        <v>547442681</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F12" s="7">
-        <v>46049</v>
+        <v>46044</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>58</v>
       </c>
       <c r="K12" s="4">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="L12" s="14">
         <f ca="1">IF($O12="","",$O12-TODAY())</f>
-        <v>-165</v>
+        <v>-170</v>
       </c>
       <c r="M12" s="14">
-        <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
-        <v>348</v>
+        <f ca="1">IF($F12="","",$F12+90-TODAY())</f>
+        <v>-170</v>
       </c>
       <c r="N12" s="14">
         <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
-        <v>348</v>
+        <v>155</v>
       </c>
       <c r="O12" s="7">
-        <v>46139</v>
+        <v>46134</v>
       </c>
       <c r="P12" s="6" t="s">
         <v>78</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="T12" s="6" t="s">
         <v>46</v>
@@ -4825,34 +4823,34 @@
         <v>976.64</v>
       </c>
       <c r="AA12" s="9">
-        <v>0</v>
+        <v>840.66</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="7">
-        <v>46133</v>
+        <v>46094</v>
       </c>
       <c r="AD12" s="9">
-        <v>976.64</v>
+        <v>135.97999999999999</v>
       </c>
       <c r="AE12" s="5">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="AF12" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AG12" s="6" t="s">
         <v>71</v>
       </c>
+      <c r="AG12" s="6"/>
       <c r="AH12" s="6"/>
       <c r="AI12" s="6"/>
-      <c r="AJ12" s="5"/>
+      <c r="AJ12" s="5">
+        <v>556556161</v>
+      </c>
       <c r="AK12" s="6" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="AL12" s="6" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="AM12" s="7">
         <v>46056</v>
@@ -4863,22 +4861,22 @@
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C13" s="4">
-        <v>46066</v>
+        <v>46128</v>
       </c>
       <c r="D13" s="5">
-        <v>547976909</v>
+        <v>555599776</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="F13" s="7">
-        <v>46051</v>
+        <v>46049</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>43</v>
@@ -4887,28 +4885,28 @@
         <v>43</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>107</v>
+        <v>76</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>58</v>
+        <v>100</v>
       </c>
       <c r="K13" s="4">
-        <v>46245</v>
+        <v>46122</v>
       </c>
       <c r="L13" s="14">
         <f ca="1">IF($O13="","",$O13-TODAY())</f>
-        <v>-163</v>
+        <v>-165</v>
       </c>
       <c r="M13" s="14">
         <f ca="1">IF($F13="","",$F13+90-TODAY())</f>
-        <v>-163</v>
+        <v>-165</v>
       </c>
       <c r="N13" s="14">
         <f ca="1">IF($C13="","",$C13+365-TODAY())</f>
-        <v>127</v>
+        <v>189</v>
       </c>
       <c r="O13" s="7">
-        <v>46141</v>
+        <v>46139</v>
       </c>
       <c r="P13" s="6" t="s">
         <v>78</v>
@@ -4935,7 +4933,7 @@
         <v>59</v>
       </c>
       <c r="Z13" s="9">
-        <v>976.64</v>
+        <v>1426.25</v>
       </c>
       <c r="AA13" s="9">
         <v>0</v>
@@ -4944,29 +4942,29 @@
         <v>0</v>
       </c>
       <c r="AC13" s="7">
-        <v>46066</v>
+        <v>46128</v>
       </c>
       <c r="AD13" s="9">
-        <v>976.64</v>
+        <v>1426.25</v>
       </c>
       <c r="AE13" s="5">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AF13" s="6" t="s">
-        <v>108</v>
+        <v>51</v>
       </c>
       <c r="AG13" s="6"/>
       <c r="AH13" s="6"/>
       <c r="AI13" s="6"/>
       <c r="AJ13" s="5"/>
       <c r="AK13" s="6" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="AL13" s="6" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="AM13" s="7">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="AN13" s="6" t="s">
         <v>54</v>
@@ -4974,58 +4972,58 @@
     </row>
     <row r="14" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>110</v>
+        <v>308</v>
       </c>
       <c r="C14" s="4">
-        <v>46098</v>
+        <v>46287</v>
       </c>
       <c r="D14" s="5">
-        <v>557090486</v>
+        <v>556349314</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="F14" s="7">
-        <v>46036</v>
+        <v>46049</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>76</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="K14" s="4">
-        <v>46135</v>
+        <v>46300</v>
       </c>
       <c r="L14" s="14">
         <f ca="1">IF($O14="","",$O14-TODAY())</f>
-        <v>-148</v>
+        <v>-165</v>
       </c>
       <c r="M14" s="14">
         <f ca="1">IF($C14="","",$C14+365-TODAY())</f>
-        <v>159</v>
+        <v>348</v>
       </c>
       <c r="N14" s="14">
-        <f ca="1">IF($C14="","",$C14+90-TODAY())</f>
-        <v>-116</v>
+        <f ca="1">IF($C14="","",$C14+365-TODAY())</f>
+        <v>348</v>
       </c>
       <c r="O14" s="7">
-        <v>46156</v>
+        <v>46139</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="R14" s="6" t="s">
         <v>46</v>
@@ -5034,7 +5032,7 @@
         <v>48</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="U14" s="6" t="s">
         <v>48</v>
@@ -5043,10 +5041,10 @@
       <c r="W14" s="6"/>
       <c r="X14" s="6"/>
       <c r="Y14" s="6" t="s">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="Z14" s="9">
-        <v>1769.18</v>
+        <v>976.64</v>
       </c>
       <c r="AA14" s="9">
         <v>0</v>
@@ -5055,26 +5053,28 @@
         <v>0</v>
       </c>
       <c r="AC14" s="7">
-        <v>46098</v>
+        <v>46133</v>
       </c>
       <c r="AD14" s="9">
-        <v>1769.18</v>
+        <v>976.64</v>
       </c>
       <c r="AE14" s="5">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="AF14" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="AG14" s="6"/>
+        <v>103</v>
+      </c>
+      <c r="AG14" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="AH14" s="6"/>
       <c r="AI14" s="6"/>
       <c r="AJ14" s="5"/>
       <c r="AK14" s="6" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="AL14" s="6" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="AM14" s="7">
         <v>46056</v>
@@ -5085,64 +5085,64 @@
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>315</v>
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="C15" s="4">
-        <v>46070</v>
+        <v>46066</v>
       </c>
       <c r="D15" s="5">
-        <v>565238310</v>
+        <v>547976909</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="F15" s="7">
-        <v>46045</v>
+        <v>46051</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="K15" s="4">
-        <v>46289</v>
+        <v>46245</v>
       </c>
       <c r="L15" s="14">
         <f ca="1">IF($O15="","",$O15-TODAY())</f>
-        <v>-79</v>
+        <v>-163</v>
       </c>
       <c r="M15" s="14">
-        <f ca="1">IF($C15="","",$C15+365-TODAY())</f>
-        <v>131</v>
+        <f ca="1">IF($F15="","",$F15+90-TODAY())</f>
+        <v>-163</v>
       </c>
       <c r="N15" s="14">
         <f ca="1">IF($C15="","",$C15+365-TODAY())</f>
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="O15" s="7">
-        <v>46225</v>
+        <v>46141</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="T15" s="6" t="s">
         <v>46</v>
@@ -5157,7 +5157,7 @@
         <v>59</v>
       </c>
       <c r="Z15" s="9">
-        <v>1426.25</v>
+        <v>976.64</v>
       </c>
       <c r="AA15" s="9">
         <v>0</v>
@@ -5166,29 +5166,29 @@
         <v>0</v>
       </c>
       <c r="AC15" s="7">
-        <v>46070</v>
+        <v>46066</v>
       </c>
       <c r="AD15" s="9">
-        <v>1426.25</v>
+        <v>976.64</v>
       </c>
       <c r="AE15" s="5">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="AF15" s="6" t="s">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="AG15" s="6"/>
       <c r="AH15" s="6"/>
       <c r="AI15" s="6"/>
       <c r="AJ15" s="5"/>
       <c r="AK15" s="6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="AL15" s="6" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="AM15" s="7">
-        <v>46057</v>
+        <v>46056</v>
       </c>
       <c r="AN15" s="6" t="s">
         <v>54</v>
@@ -10394,7 +10394,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>305</v>
       </c>

</xml_diff>